<commit_message>
T3.2 - Avaliação Heurística
</commit_message>
<xml_diff>
--- a/T3/AvaliacaoHeuristica.xlsx
+++ b/T3/AvaliacaoHeuristica.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Experiencia_do_Usuario\T3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B33CC62-40BD-4F0B-AF68-AFC7ED2E059F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF5F46C9-F569-4491-86C1-3644CCA4B8A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="16200" activeTab="1" xr2:uid="{C5DD57C8-0B84-458E-9237-08286E66ECD5}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="11835" activeTab="1" xr2:uid="{C5DD57C8-0B84-458E-9237-08286E66ECD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Carolina Ferreira" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="32">
   <si>
     <t>Tela Principal</t>
   </si>
@@ -111,6 +111,51 @@
   </si>
   <si>
     <t>2. Talvez usar mais icones nos filtros</t>
+  </si>
+  <si>
+    <t>ObsII: Nota 0 = Não há problemas com a heurística em questão</t>
+  </si>
+  <si>
+    <t>ObsIII: Nota - = Heurística não se aplica</t>
+  </si>
+  <si>
+    <t>ObsI: Notas em escala 1-9 em relação a quão problemática/ausente está a heurística em questão</t>
+  </si>
+  <si>
+    <t>3. Protótipo não demonstra possibilidade de apagar mensagens enviadas incorretamente</t>
+  </si>
+  <si>
+    <t>3. Não há um botão claro para anular os filtros</t>
+  </si>
+  <si>
+    <t>3. Não é necessariamente claro como desmarcar presença no evento</t>
+  </si>
+  <si>
+    <t>3. Talvez possibilidade de desfazer uma avaliação</t>
+  </si>
+  <si>
+    <t>*5 para todos: Não há interfaces definidas de confirmação para nada</t>
+  </si>
+  <si>
+    <t>6. Instrução de como confirmar presença</t>
+  </si>
+  <si>
+    <t>7. Não há nenhum acelerador de filtros</t>
+  </si>
+  <si>
+    <t>8. Não sei se o nome do Host é relevante noos outrros eventos</t>
+  </si>
+  <si>
+    <t>*9 para todos: Não há previsão de mensagens de erro</t>
+  </si>
+  <si>
+    <t>10. Um botão de ajuda/FAQ ao lado das notificações poderia ajudar</t>
+  </si>
+  <si>
+    <t>10. Prever textos auxiliares na hora da avaliação</t>
+  </si>
+  <si>
+    <t>10. Prever interface de ajuda ao pressionar um botão talvez</t>
   </si>
 </sst>
 </file>
@@ -778,7 +823,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C098EFD-D4EB-420E-B5AD-D50319D83283}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
@@ -789,7 +834,7 @@
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
@@ -809,7 +854,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -828,12 +873,17 @@
       <c r="F2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="1"/>
+      <c r="B3" s="1">
+        <v>0</v>
+      </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
@@ -846,106 +896,231 @@
       <c r="F3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1">
+        <v>3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>3</v>
+      </c>
+      <c r="H6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
+        <v>2</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1">
+        <v>3</v>
+      </c>
+      <c r="E10" s="1">
+        <v>3</v>
+      </c>
+      <c r="F10" s="1">
+        <v>3</v>
+      </c>
+      <c r="H10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" s="5" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="B12" s="6"/>
+      <c r="B11" s="1">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="5" customFormat="1" ht="120" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>29</v>
+      </c>
       <c r="C12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="E12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="6"/>
-    </row>
-    <row r="13" spans="1:6" s="5" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F12" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="5" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="C13" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+      <c r="D13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="5" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="C14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="5" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+      <c r="C15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="5" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+      <c r="E16" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
     <row r="17" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="18" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="19" s="5" customFormat="1" x14ac:dyDescent="0.25"/>

</xml_diff>